<commit_message>
updated python excel file
</commit_message>
<xml_diff>
--- a/CAP766(PYTHON).xlsx
+++ b/CAP766(PYTHON).xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Desktop\776\CAP776-GROUP-I-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EDC46701-1B81-4C29-855E-9FC46B1FF73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC35C866-84FB-4BEB-B8EC-D536D8581994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="113" uniqueCount="71">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -227,6 +227,18 @@
   </si>
   <si>
     <t>productive day.</t>
+  </si>
+  <si>
+    <t>quite good.</t>
+  </si>
+  <si>
+    <t>it was a good day.</t>
+  </si>
+  <si>
+    <t>unique day it was.</t>
+  </si>
+  <si>
+    <t>had regular classes and completed a little study at night.</t>
   </si>
 </sst>
 </file>
@@ -1468,114 +1480,234 @@
       </c>
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A16" s="13"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14"/>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="14"/>
-      <c r="I16" s="15" t="str">
+      <c r="A16" s="13">
+        <v>46256</v>
+      </c>
+      <c r="B16" s="14">
+        <v>300</v>
+      </c>
+      <c r="C16" s="14">
+        <v>20</v>
+      </c>
+      <c r="D16" s="14">
+        <v>150</v>
+      </c>
+      <c r="E16" s="14">
+        <v>20</v>
+      </c>
+      <c r="F16" s="14">
+        <v>0</v>
+      </c>
+      <c r="G16" s="14">
+        <v>0</v>
+      </c>
+      <c r="H16" s="14">
+        <v>120</v>
+      </c>
+      <c r="I16" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="15" t="str">
+        <v>610</v>
+      </c>
+      <c r="J16" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K16" s="16"/>
-      <c r="L16" s="16"/>
-      <c r="M16" s="16"/>
-      <c r="N16" s="17"/>
+        <v>830</v>
+      </c>
+      <c r="K16" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L16" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M16" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N16" s="17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A17" s="13"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="15" t="str">
+      <c r="A17" s="13">
+        <v>46257</v>
+      </c>
+      <c r="B17" s="14">
+        <v>360</v>
+      </c>
+      <c r="C17" s="14">
+        <v>0</v>
+      </c>
+      <c r="D17" s="14">
+        <v>120</v>
+      </c>
+      <c r="E17" s="14">
+        <v>25</v>
+      </c>
+      <c r="F17" s="14">
+        <v>0</v>
+      </c>
+      <c r="G17" s="14">
+        <v>0</v>
+      </c>
+      <c r="H17" s="14">
+        <v>120</v>
+      </c>
+      <c r="I17" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="15" t="str">
+        <v>625</v>
+      </c>
+      <c r="J17" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K17" s="16"/>
-      <c r="L17" s="16"/>
-      <c r="M17" s="16"/>
-      <c r="N17" s="17"/>
+        <v>815</v>
+      </c>
+      <c r="K17" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L17" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M17" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N17" s="17" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A18" s="13"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
-      <c r="I18" s="15" t="str">
+      <c r="A18" s="13">
+        <v>46258</v>
+      </c>
+      <c r="B18" s="14">
+        <v>420</v>
+      </c>
+      <c r="C18" s="14">
+        <v>20</v>
+      </c>
+      <c r="D18" s="14">
+        <v>120</v>
+      </c>
+      <c r="E18" s="14">
+        <v>45</v>
+      </c>
+      <c r="F18" s="14">
+        <v>100</v>
+      </c>
+      <c r="G18" s="14">
+        <v>2</v>
+      </c>
+      <c r="H18" s="14">
+        <v>60</v>
+      </c>
+      <c r="I18" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="15" t="str">
+        <v>765</v>
+      </c>
+      <c r="J18" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K18" s="16"/>
-      <c r="L18" s="16"/>
-      <c r="M18" s="16"/>
-      <c r="N18" s="17"/>
+        <v>675</v>
+      </c>
+      <c r="K18" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L18" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M18" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N18" s="17" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A19" s="13"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
-      <c r="I19" s="15" t="str">
+      <c r="A19" s="13">
+        <v>46259</v>
+      </c>
+      <c r="B19" s="14">
+        <v>300</v>
+      </c>
+      <c r="C19" s="14">
+        <v>25</v>
+      </c>
+      <c r="D19" s="14">
+        <v>150</v>
+      </c>
+      <c r="E19" s="14">
+        <v>60</v>
+      </c>
+      <c r="F19" s="14">
+        <v>350</v>
+      </c>
+      <c r="G19" s="14">
+        <v>7</v>
+      </c>
+      <c r="H19" s="14">
+        <v>120</v>
+      </c>
+      <c r="I19" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
+        <v>1005</v>
+      </c>
+      <c r="J19" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K19" s="16"/>
-      <c r="L19" s="16"/>
-      <c r="M19" s="16"/>
-      <c r="N19" s="17"/>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A20" s="13"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
-      <c r="I20" s="15" t="str">
+        <v>435</v>
+      </c>
+      <c r="K19" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L19" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M19" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N19" s="17" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A20" s="13">
+        <v>46260</v>
+      </c>
+      <c r="B20" s="14">
+        <v>300</v>
+      </c>
+      <c r="C20" s="14">
+        <v>40</v>
+      </c>
+      <c r="D20" s="14">
+        <v>120</v>
+      </c>
+      <c r="E20" s="14">
+        <v>20</v>
+      </c>
+      <c r="F20" s="14">
+        <v>200</v>
+      </c>
+      <c r="G20" s="14">
+        <v>4</v>
+      </c>
+      <c r="H20" s="14">
+        <v>180</v>
+      </c>
+      <c r="I20" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
+        <v>860</v>
+      </c>
+      <c r="J20" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K20" s="16"/>
-      <c r="L20" s="16"/>
-      <c r="M20" s="16"/>
-      <c r="N20" s="17"/>
+        <v>580</v>
+      </c>
+      <c r="K20" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L20" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="M20" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N20" s="17" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A21" s="13"/>

</xml_diff>

<commit_message>
updated excel file sheet
</commit_message>
<xml_diff>
--- a/CAP766(PYTHON).xlsx
+++ b/CAP766(PYTHON).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\asus\Desktop\776\CAP776-GROUP-I-\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81275916-5B2D-4E17-A82D-EAA0844FF906}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{527628D5-CDF7-4CF9-96A6-992A538C8B1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="78">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -256,7 +256,10 @@
     <t>felt a bit tired after evening classes.</t>
   </si>
   <si>
-    <t>I have done my frist presenation on Topic in PEL class.</t>
+    <t>I have done my first presenation on a Topic in PEL class.</t>
+  </si>
+  <si>
+    <t>good day.</t>
   </si>
 </sst>
 </file>
@@ -443,7 +446,31 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="3">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+        <name val="Arial"/>
+        <charset val="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -2050,29 +2077,55 @@
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A28" s="13"/>
-      <c r="B28" s="14"/>
-      <c r="C28" s="14"/>
-      <c r="D28" s="14"/>
-      <c r="E28" s="14"/>
-      <c r="F28" s="14"/>
-      <c r="G28" s="14"/>
-      <c r="H28" s="14"/>
-      <c r="I28" s="15" t="str">
+      <c r="A28" s="13">
+        <v>46268</v>
+      </c>
+      <c r="B28" s="14">
+        <v>360</v>
+      </c>
+      <c r="C28" s="14">
+        <v>40</v>
+      </c>
+      <c r="D28" s="14">
+        <v>180</v>
+      </c>
+      <c r="E28" s="14">
+        <v>30</v>
+      </c>
+      <c r="F28" s="14">
+        <v>350</v>
+      </c>
+      <c r="G28" s="14">
+        <v>7</v>
+      </c>
+      <c r="H28" s="14">
+        <v>120</v>
+      </c>
+      <c r="I28" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J28" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K28" s="16"/>
-      <c r="L28" s="16"/>
-      <c r="M28" s="16"/>
-      <c r="N28" s="17"/>
+        <v>360</v>
+      </c>
+      <c r="K28" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L28" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M28" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N28" s="17" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A29" s="13"/>
+      <c r="A29" s="13">
+        <v>46269</v>
+      </c>
       <c r="B29" s="14"/>
       <c r="C29" s="14"/>
       <c r="D29" s="14"/>
@@ -10286,8 +10339,13 @@
     <mergeCell ref="B3:D3"/>
     <mergeCell ref="F3:G3"/>
   </mergeCells>
-  <conditionalFormatting sqref="J6:J401">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="lessThan">
+  <conditionalFormatting sqref="J6:J27 J29:J401">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J28">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>